<commit_message>
Suppression partie concil et dispense d4360184a8570403b8850c1aaa422b35aead4d14
</commit_message>
<xml_diff>
--- a/Finalisation-concertation/ig/CodeSystem-fr-additional-action-relationship-type.xlsx
+++ b/Finalisation-concertation/ig/CodeSystem-fr-additional-action-relationship-type.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>https://hl7.fr/ig/fhir/medication/CodeSystem/fr-additional-action-relationship-type</t>
+    <t>https://hl7.fr/ig/fhir/analyse-pharma/CodeSystem/fr-additional-action-relationship-type</t>
   </si>
   <si>
     <t>Version</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-21T12:38:31+00:00</t>
+    <t>2026-05-21T13:21:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>